<commit_message>
Preprocess once for both outputs: equal row counts, Antioquia fallback, silent dedup
- Deduplication happens once before building campaign and customers,
  guaranteeing identical row counts between paired files
- Duplicates silently dropped; bad-phone rows still route to .review
- voice_model_selection falls back to 'Antioquia' when phone not in template
</commit_message>
<xml_diff>
--- a/output/customers_Vive_Living.xlsx
+++ b/output/customers_Vive_Living.xlsx
@@ -459,8 +459,10 @@
           <t>Berrios Olivera</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -479,8 +481,10 @@
           <t>Arango Ossa</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -499,8 +503,10 @@
           <t>Gaviria Hernandez</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -519,8 +525,10 @@
           <t>Garzón</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -539,8 +547,10 @@
           <t>Otero</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -559,8 +569,10 @@
           <t>Ramirez Díaz</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -579,8 +591,10 @@
           <t>Molina</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -599,8 +613,10 @@
           <t>Medina</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -619,8 +635,10 @@
           <t>Ome</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -639,8 +657,10 @@
           <t>Ramirez Atehortúa</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -659,8 +679,10 @@
           <t>Moreno</t>
         </is>
       </c>
-      <c r="E12" t="n">
-        <v/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -679,8 +701,10 @@
           <t>Gomez</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -699,8 +723,10 @@
           <t>Bocanegra</t>
         </is>
       </c>
-      <c r="E14" t="n">
-        <v/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -719,8 +745,10 @@
           <t>Hincapie</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -739,8 +767,10 @@
           <t>Abdala Gonzalez</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -759,8 +789,10 @@
           <t>Álvarez</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -779,8 +811,10 @@
           <t>Alcalá Quijano</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -799,8 +833,10 @@
           <t>Serna</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -819,8 +855,10 @@
           <t>Malaver</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -839,8 +877,10 @@
           <t>Cadavid</t>
         </is>
       </c>
-      <c r="E21" t="n">
-        <v/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -859,8 +899,10 @@
           <t>Lopez</t>
         </is>
       </c>
-      <c r="E22" t="n">
-        <v/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -879,8 +921,10 @@
           <t>Torres</t>
         </is>
       </c>
-      <c r="E23" t="n">
-        <v/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -899,8 +943,10 @@
           <t>Torres</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -919,8 +965,10 @@
           <t>Ayala Lopez</t>
         </is>
       </c>
-      <c r="E25" t="n">
-        <v/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -939,8 +987,10 @@
           <t>Naranjo</t>
         </is>
       </c>
-      <c r="E26" t="n">
-        <v/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -959,8 +1009,10 @@
           <t>Gomez</t>
         </is>
       </c>
-      <c r="E27" t="n">
-        <v/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -979,8 +1031,10 @@
           <t>Longa</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -999,8 +1053,10 @@
           <t>Manco Tobon</t>
         </is>
       </c>
-      <c r="E29" t="n">
-        <v/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1019,8 +1075,10 @@
           <t>Bernal</t>
         </is>
       </c>
-      <c r="E30" t="n">
-        <v/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -1039,8 +1097,10 @@
           <t>Mora</t>
         </is>
       </c>
-      <c r="E31" t="n">
-        <v/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -1059,8 +1119,10 @@
           <t>Ramirez</t>
         </is>
       </c>
-      <c r="E32" t="n">
-        <v/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1101,8 +1163,10 @@
           <t>Morales</t>
         </is>
       </c>
-      <c r="E34" t="n">
-        <v/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -1121,8 +1185,10 @@
           <t>Restrepo</t>
         </is>
       </c>
-      <c r="E35" t="n">
-        <v/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -1141,8 +1207,10 @@
           <t>Marcela</t>
         </is>
       </c>
-      <c r="E36" t="n">
-        <v/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -1161,8 +1229,10 @@
           <t>Duran</t>
         </is>
       </c>
-      <c r="E37" t="n">
-        <v/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1181,8 +1251,10 @@
           <t>Perez</t>
         </is>
       </c>
-      <c r="E38" t="n">
-        <v/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -1201,8 +1273,10 @@
           <t>Mosquera Vanegas</t>
         </is>
       </c>
-      <c r="E39" t="n">
-        <v/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -1221,8 +1295,10 @@
           <t>Parra</t>
         </is>
       </c>
-      <c r="E40" t="n">
-        <v/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -1241,8 +1317,10 @@
           <t>Mejia</t>
         </is>
       </c>
-      <c r="E41" t="n">
-        <v/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -1261,8 +1339,10 @@
           <t>Espinosa</t>
         </is>
       </c>
-      <c r="E42" t="n">
-        <v/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -1281,8 +1361,10 @@
           <t>Mendez</t>
         </is>
       </c>
-      <c r="E43" t="n">
-        <v/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -1301,8 +1383,10 @@
           <t>Villa Villegas</t>
         </is>
       </c>
-      <c r="E44" t="n">
-        <v/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -1321,8 +1405,10 @@
           <t>Calle</t>
         </is>
       </c>
-      <c r="E45" t="n">
-        <v/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -1341,8 +1427,10 @@
           <t>Gomez</t>
         </is>
       </c>
-      <c r="E46" t="n">
-        <v/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -1361,8 +1449,10 @@
           <t>Barrera</t>
         </is>
       </c>
-      <c r="E47" t="n">
-        <v/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -1381,8 +1471,10 @@
           <t>Londoño Castaño</t>
         </is>
       </c>
-      <c r="E48" t="n">
-        <v/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -1401,8 +1493,10 @@
           <t>Lopez</t>
         </is>
       </c>
-      <c r="E49" t="n">
-        <v/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -1421,8 +1515,10 @@
           <t>Garcia</t>
         </is>
       </c>
-      <c r="E50" t="n">
-        <v/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -1441,8 +1537,10 @@
           <t>Zambrano</t>
         </is>
       </c>
-      <c r="E51" t="n">
-        <v/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -1461,8 +1559,10 @@
           <t>Rodriguez</t>
         </is>
       </c>
-      <c r="E52" t="n">
-        <v/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -1481,8 +1581,10 @@
           <t>Cardenas Cruz</t>
         </is>
       </c>
-      <c r="E53" t="n">
-        <v/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -1501,8 +1603,10 @@
           <t>Zapata</t>
         </is>
       </c>
-      <c r="E54" t="n">
-        <v/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -1521,8 +1625,10 @@
           <t>Montaño Parra</t>
         </is>
       </c>
-      <c r="E55" t="n">
-        <v/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -1541,8 +1647,10 @@
           <t>Arboleda</t>
         </is>
       </c>
-      <c r="E56" t="n">
-        <v/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -1583,8 +1691,10 @@
           <t>Lopera Velez</t>
         </is>
       </c>
-      <c r="E58" t="n">
-        <v/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -1603,8 +1713,10 @@
           <t>Mejia</t>
         </is>
       </c>
-      <c r="E59" t="n">
-        <v/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -1623,8 +1735,10 @@
           <t>Herrera</t>
         </is>
       </c>
-      <c r="E60" t="n">
-        <v/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -1643,8 +1757,10 @@
           <t>Cano</t>
         </is>
       </c>
-      <c r="E61" t="n">
-        <v/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -1663,8 +1779,10 @@
           <t>Mejia</t>
         </is>
       </c>
-      <c r="E62" t="n">
-        <v/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -1705,8 +1823,10 @@
           <t>Restrepo</t>
         </is>
       </c>
-      <c r="E64" t="n">
-        <v/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -1725,8 +1845,10 @@
           <t>Castano</t>
         </is>
       </c>
-      <c r="E65" t="n">
-        <v/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -1745,8 +1867,10 @@
           <t>Duque</t>
         </is>
       </c>
-      <c r="E66" t="n">
-        <v/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -1765,8 +1889,10 @@
           <t>Freydell</t>
         </is>
       </c>
-      <c r="E67" t="n">
-        <v/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -1785,8 +1911,10 @@
           <t>Serna Blandon</t>
         </is>
       </c>
-      <c r="E68" t="n">
-        <v/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -1805,8 +1933,10 @@
           <t>Lasso Arias</t>
         </is>
       </c>
-      <c r="E69" t="n">
-        <v/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -1825,8 +1955,10 @@
           <t>Chico Torres</t>
         </is>
       </c>
-      <c r="E70" t="n">
-        <v/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -1845,8 +1977,10 @@
           <t>Gutierrez Rivas</t>
         </is>
       </c>
-      <c r="E71" t="n">
-        <v/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -1865,8 +1999,10 @@
           <t>Villegas</t>
         </is>
       </c>
-      <c r="E72" t="n">
-        <v/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -1885,8 +2021,10 @@
           <t>Bermudez</t>
         </is>
       </c>
-      <c r="E73" t="n">
-        <v/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -1905,8 +2043,10 @@
           <t>Roldán Botero</t>
         </is>
       </c>
-      <c r="E74" t="n">
-        <v/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -1925,8 +2065,10 @@
           <t>Jiménez</t>
         </is>
       </c>
-      <c r="E75" t="n">
-        <v/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -1945,8 +2087,10 @@
           <t>Acosta</t>
         </is>
       </c>
-      <c r="E76" t="n">
-        <v/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="77">
@@ -1965,8 +2109,10 @@
           <t>Vélez</t>
         </is>
       </c>
-      <c r="E77" t="n">
-        <v/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -1985,8 +2131,10 @@
           <t>Escobar Vélez</t>
         </is>
       </c>
-      <c r="E78" t="n">
-        <v/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -2005,8 +2153,10 @@
           <t>Patiño</t>
         </is>
       </c>
-      <c r="E79" t="n">
-        <v/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -2025,8 +2175,10 @@
           <t>Becerra</t>
         </is>
       </c>
-      <c r="E80" t="n">
-        <v/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -2045,8 +2197,10 @@
           <t>Montoya Hoyos</t>
         </is>
       </c>
-      <c r="E81" t="n">
-        <v/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -2065,8 +2219,10 @@
           <t>Sánchez</t>
         </is>
       </c>
-      <c r="E82" t="n">
-        <v/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="83">
@@ -2085,8 +2241,10 @@
           <t>Gaviria</t>
         </is>
       </c>
-      <c r="E83" t="n">
-        <v/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="84">
@@ -2105,8 +2263,10 @@
           <t>Matiz</t>
         </is>
       </c>
-      <c r="E84" t="n">
-        <v/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -2125,8 +2285,10 @@
           <t>Cortes Santos</t>
         </is>
       </c>
-      <c r="E85" t="n">
-        <v/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="86">
@@ -2145,8 +2307,10 @@
           <t>Vargas</t>
         </is>
       </c>
-      <c r="E86" t="n">
-        <v/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="87">
@@ -2165,8 +2329,10 @@
           <t>Hincapi</t>
         </is>
       </c>
-      <c r="E87" t="n">
-        <v/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="88">
@@ -2185,8 +2351,10 @@
           <t>Segura</t>
         </is>
       </c>
-      <c r="E88" t="n">
-        <v/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="89">
@@ -2205,8 +2373,10 @@
           <t>Daza</t>
         </is>
       </c>
-      <c r="E89" t="n">
-        <v/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="90">
@@ -2225,8 +2395,10 @@
           <t>Patiño</t>
         </is>
       </c>
-      <c r="E90" t="n">
-        <v/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="91">
@@ -2245,8 +2417,10 @@
           <t>Moreno</t>
         </is>
       </c>
-      <c r="E91" t="n">
-        <v/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="92">
@@ -2265,8 +2439,10 @@
           <t>Fajardo</t>
         </is>
       </c>
-      <c r="E92" t="n">
-        <v/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="93">
@@ -2285,8 +2461,10 @@
           <t>Mejia Gomez</t>
         </is>
       </c>
-      <c r="E93" t="n">
-        <v/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="94">
@@ -2305,8 +2483,10 @@
           <t>Espinal</t>
         </is>
       </c>
-      <c r="E94" t="n">
-        <v/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="95">
@@ -2325,8 +2505,10 @@
           <t>Vlez</t>
         </is>
       </c>
-      <c r="E95" t="n">
-        <v/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="96">
@@ -2345,8 +2527,10 @@
           <t>Lovera</t>
         </is>
       </c>
-      <c r="E96" t="n">
-        <v/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="97">
@@ -2365,8 +2549,10 @@
           <t>Orozco</t>
         </is>
       </c>
-      <c r="E97" t="n">
-        <v/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="98">
@@ -2385,8 +2571,10 @@
           <t>Franco</t>
         </is>
       </c>
-      <c r="E98" t="n">
-        <v/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="99">
@@ -2405,8 +2593,10 @@
           <t>Ramirez</t>
         </is>
       </c>
-      <c r="E99" t="n">
-        <v/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="100">
@@ -2425,8 +2615,10 @@
           <t>Herrera Herrera</t>
         </is>
       </c>
-      <c r="E100" t="n">
-        <v/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="101">
@@ -2445,8 +2637,10 @@
           <t>Salazar Arredondo</t>
         </is>
       </c>
-      <c r="E101" t="n">
-        <v/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="102">
@@ -2465,8 +2659,10 @@
           <t>Rios</t>
         </is>
       </c>
-      <c r="E102" t="n">
-        <v/>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="103">
@@ -2485,8 +2681,10 @@
           <t>Ramirez</t>
         </is>
       </c>
-      <c r="E103" t="n">
-        <v/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="104">
@@ -2505,8 +2703,10 @@
           <t>Marin Osorio</t>
         </is>
       </c>
-      <c r="E104" t="n">
-        <v/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="105">
@@ -2525,8 +2725,10 @@
           <t>Vélez</t>
         </is>
       </c>
-      <c r="E105" t="n">
-        <v/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="106">
@@ -2545,8 +2747,10 @@
           <t>Saldarriaga</t>
         </is>
       </c>
-      <c r="E106" t="n">
-        <v/>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="107">
@@ -2565,8 +2769,10 @@
           <t>Gil</t>
         </is>
       </c>
-      <c r="E107" t="n">
-        <v/>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="108">
@@ -2585,8 +2791,10 @@
           <t>Rodriguez</t>
         </is>
       </c>
-      <c r="E108" t="n">
-        <v/>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="109">
@@ -2605,8 +2813,10 @@
           <t>Gómez Fernández</t>
         </is>
       </c>
-      <c r="E109" t="n">
-        <v/>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="110">
@@ -2625,8 +2835,10 @@
           <t>Alvarez</t>
         </is>
       </c>
-      <c r="E110" t="n">
-        <v/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="111">
@@ -2645,8 +2857,10 @@
           <t>Quintero</t>
         </is>
       </c>
-      <c r="E111" t="n">
-        <v/>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="112">
@@ -2665,8 +2879,10 @@
           <t>Martinez</t>
         </is>
       </c>
-      <c r="E112" t="n">
-        <v/>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="113">
@@ -2685,8 +2901,10 @@
           <t>Villa</t>
         </is>
       </c>
-      <c r="E113" t="n">
-        <v/>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="114">
@@ -2705,8 +2923,10 @@
           <t>Montoya</t>
         </is>
       </c>
-      <c r="E114" t="n">
-        <v/>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="115">
@@ -2725,8 +2945,10 @@
           <t>Mueses</t>
         </is>
       </c>
-      <c r="E115" t="n">
-        <v/>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="116">
@@ -2745,8 +2967,10 @@
           <t>Echavarria</t>
         </is>
       </c>
-      <c r="E116" t="n">
-        <v/>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="117">
@@ -2765,8 +2989,10 @@
           <t>Turpin Martinez</t>
         </is>
       </c>
-      <c r="E117" t="n">
-        <v/>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="118">
@@ -2785,8 +3011,10 @@
           <t>Espinosa Montoya</t>
         </is>
       </c>
-      <c r="E118" t="n">
-        <v/>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="119">
@@ -2805,8 +3033,10 @@
           <t>Tobías</t>
         </is>
       </c>
-      <c r="E119" t="n">
-        <v/>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="120">
@@ -2825,8 +3055,10 @@
           <t>Botia</t>
         </is>
       </c>
-      <c r="E120" t="n">
-        <v/>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="121">
@@ -2845,8 +3077,10 @@
           <t>Quiintero</t>
         </is>
       </c>
-      <c r="E121" t="n">
-        <v/>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="122">
@@ -2865,8 +3099,10 @@
           <t>Mejia Restrepo</t>
         </is>
       </c>
-      <c r="E122" t="n">
-        <v/>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="123">
@@ -2885,8 +3121,10 @@
           <t>Gutierrez Giraldo</t>
         </is>
       </c>
-      <c r="E123" t="n">
-        <v/>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="124">
@@ -2905,8 +3143,10 @@
           <t>Hernández Camargo</t>
         </is>
       </c>
-      <c r="E124" t="n">
-        <v/>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="125">
@@ -2925,8 +3165,10 @@
           <t>Restrepo Correa</t>
         </is>
       </c>
-      <c r="E125" t="n">
-        <v/>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="126">
@@ -2945,8 +3187,10 @@
           <t>Uribe</t>
         </is>
       </c>
-      <c r="E126" t="n">
-        <v/>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="127">
@@ -2965,8 +3209,10 @@
           <t>Zuluaga Salazar</t>
         </is>
       </c>
-      <c r="E127" t="n">
-        <v/>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="128">
@@ -2985,8 +3231,10 @@
           <t>Gutierrez Garcia</t>
         </is>
       </c>
-      <c r="E128" t="n">
-        <v/>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="129">
@@ -3005,8 +3253,10 @@
           <t>Pelaez</t>
         </is>
       </c>
-      <c r="E129" t="n">
-        <v/>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="130">
@@ -3025,8 +3275,10 @@
           <t>Pérez</t>
         </is>
       </c>
-      <c r="E130" t="n">
-        <v/>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="131">
@@ -3045,8 +3297,10 @@
           <t>Gómez</t>
         </is>
       </c>
-      <c r="E131" t="n">
-        <v/>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="132">
@@ -3065,8 +3319,10 @@
           <t>Rincón Castaño</t>
         </is>
       </c>
-      <c r="E132" t="n">
-        <v/>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="133">
@@ -3085,8 +3341,10 @@
           <t>Campo</t>
         </is>
       </c>
-      <c r="E133" t="n">
-        <v/>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="134">
@@ -3105,8 +3363,10 @@
           <t>Palacio Agudelo</t>
         </is>
       </c>
-      <c r="E134" t="n">
-        <v/>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="135">
@@ -3147,8 +3407,10 @@
           <t>Agámez Marchena</t>
         </is>
       </c>
-      <c r="E136" t="n">
-        <v/>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="137">
@@ -3167,8 +3429,10 @@
           <t>Castro</t>
         </is>
       </c>
-      <c r="E137" t="n">
-        <v/>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="138">
@@ -3187,8 +3451,10 @@
           <t>Gallego</t>
         </is>
       </c>
-      <c r="E138" t="n">
-        <v/>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="139">
@@ -3207,8 +3473,10 @@
           <t>Gutierrez Fonseca</t>
         </is>
       </c>
-      <c r="E139" t="n">
-        <v/>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="140">
@@ -3227,8 +3495,10 @@
           <t>Urueta</t>
         </is>
       </c>
-      <c r="E140" t="n">
-        <v/>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="141">
@@ -3247,8 +3517,10 @@
           <t>Grajales Rua</t>
         </is>
       </c>
-      <c r="E141" t="n">
-        <v/>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="142">
@@ -3267,8 +3539,10 @@
           <t>Hernandez</t>
         </is>
       </c>
-      <c r="E142" t="n">
-        <v/>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="143">
@@ -3287,8 +3561,10 @@
           <t>Cecilia Restrepo Alvarez</t>
         </is>
       </c>
-      <c r="E143" t="n">
-        <v/>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="144">
@@ -3307,8 +3583,10 @@
           <t>Rodriguez Zamora</t>
         </is>
       </c>
-      <c r="E144" t="n">
-        <v/>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="145">
@@ -3327,8 +3605,10 @@
           <t>Pantoja Santacruz</t>
         </is>
       </c>
-      <c r="E145" t="n">
-        <v/>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="146">
@@ -3347,8 +3627,10 @@
           <t>Trujillo</t>
         </is>
       </c>
-      <c r="E146" t="n">
-        <v/>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="147">
@@ -3367,8 +3649,10 @@
           <t>Garciagarcia</t>
         </is>
       </c>
-      <c r="E147" t="n">
-        <v/>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="148">
@@ -3387,8 +3671,10 @@
           <t>Velez Alvarez</t>
         </is>
       </c>
-      <c r="E148" t="n">
-        <v/>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="149">
@@ -3407,8 +3693,10 @@
           <t>Loboa Caicedo</t>
         </is>
       </c>
-      <c r="E149" t="n">
-        <v/>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="150">
@@ -3427,8 +3715,10 @@
           <t>Gómez Escorcia</t>
         </is>
       </c>
-      <c r="E150" t="n">
-        <v/>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="151">
@@ -3447,8 +3737,10 @@
           <t>V</t>
         </is>
       </c>
-      <c r="E151" t="n">
-        <v/>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="152">
@@ -3467,8 +3759,10 @@
           <t>Hoyos Gomez</t>
         </is>
       </c>
-      <c r="E152" t="n">
-        <v/>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="153">
@@ -3487,8 +3781,10 @@
           <t>Gonzalez</t>
         </is>
       </c>
-      <c r="E153" t="n">
-        <v/>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="154">
@@ -3507,8 +3803,10 @@
           <t>Rendon</t>
         </is>
       </c>
-      <c r="E154" t="n">
-        <v/>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="155">
@@ -3527,8 +3825,10 @@
           <t>Mario Pérez</t>
         </is>
       </c>
-      <c r="E155" t="n">
-        <v/>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="156">
@@ -3547,8 +3847,10 @@
           <t>Suescún Bedoya</t>
         </is>
       </c>
-      <c r="E156" t="n">
-        <v/>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="157">
@@ -3567,8 +3869,10 @@
           <t>Cardeño Rengifo</t>
         </is>
       </c>
-      <c r="E157" t="n">
-        <v/>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="158">
@@ -3587,8 +3891,10 @@
           <t>Contreras</t>
         </is>
       </c>
-      <c r="E158" t="n">
-        <v/>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="159">
@@ -3607,8 +3913,10 @@
           <t>Bohorquez Orozco</t>
         </is>
       </c>
-      <c r="E159" t="n">
-        <v/>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="160">
@@ -3627,8 +3935,10 @@
           <t>Hernández Castro</t>
         </is>
       </c>
-      <c r="E160" t="n">
-        <v/>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="161">
@@ -3647,8 +3957,10 @@
           <t>Bolívar</t>
         </is>
       </c>
-      <c r="E161" t="n">
-        <v/>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="162">
@@ -3667,8 +3979,10 @@
           <t>D. Arboleda</t>
         </is>
       </c>
-      <c r="E162" t="n">
-        <v/>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="163">
@@ -3687,8 +4001,10 @@
           <t>Zuluaga</t>
         </is>
       </c>
-      <c r="E163" t="n">
-        <v/>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="164">
@@ -3707,8 +4023,10 @@
           <t>Gallego Diaz</t>
         </is>
       </c>
-      <c r="E164" t="n">
-        <v/>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="165">
@@ -3727,8 +4045,10 @@
           <t>Uribe</t>
         </is>
       </c>
-      <c r="E165" t="n">
-        <v/>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="166">
@@ -3747,8 +4067,10 @@
           <t>Henao</t>
         </is>
       </c>
-      <c r="E166" t="n">
-        <v/>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="167">
@@ -3767,8 +4089,10 @@
           <t>Pnl</t>
         </is>
       </c>
-      <c r="E167" t="n">
-        <v/>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="168">
@@ -3787,8 +4111,10 @@
           <t>Mesa</t>
         </is>
       </c>
-      <c r="E168" t="n">
-        <v/>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="169">
@@ -3829,8 +4155,10 @@
           <t>Serna</t>
         </is>
       </c>
-      <c r="E170" t="n">
-        <v/>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="171">
@@ -3849,8 +4177,10 @@
           <t>Rubin</t>
         </is>
       </c>
-      <c r="E171" t="n">
-        <v/>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="172">
@@ -3869,8 +4199,10 @@
           <t>Uriana</t>
         </is>
       </c>
-      <c r="E172" t="n">
-        <v/>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="173">
@@ -3911,8 +4243,10 @@
           <t>Pareja</t>
         </is>
       </c>
-      <c r="E174" t="n">
-        <v/>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="175">
@@ -3931,8 +4265,10 @@
           <t>Molina</t>
         </is>
       </c>
-      <c r="E175" t="n">
-        <v/>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="176">
@@ -3951,8 +4287,10 @@
           <t>Hoyos</t>
         </is>
       </c>
-      <c r="E176" t="n">
-        <v/>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="177">
@@ -3971,8 +4309,10 @@
           <t>Rodriguez</t>
         </is>
       </c>
-      <c r="E177" t="n">
-        <v/>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="178">
@@ -3991,8 +4331,10 @@
           <t>Escobar</t>
         </is>
       </c>
-      <c r="E178" t="n">
-        <v/>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="179">
@@ -4011,8 +4353,10 @@
           <t>Rua Penagos</t>
         </is>
       </c>
-      <c r="E179" t="n">
-        <v/>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="180">
@@ -4031,8 +4375,10 @@
           <t>Almanza</t>
         </is>
       </c>
-      <c r="E180" t="n">
-        <v/>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="181">
@@ -4051,8 +4397,10 @@
           <t>Velasquez Giraldo</t>
         </is>
       </c>
-      <c r="E181" t="n">
-        <v/>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="182">
@@ -4093,8 +4441,10 @@
           <t>De La Hoz Osorio</t>
         </is>
       </c>
-      <c r="E183" t="n">
-        <v/>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="184">
@@ -4113,8 +4463,10 @@
           <t>Pineda Arango</t>
         </is>
       </c>
-      <c r="E184" t="n">
-        <v/>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="185">
@@ -4133,8 +4485,10 @@
           <t>Hinestrosa</t>
         </is>
       </c>
-      <c r="E185" t="n">
-        <v/>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="186">
@@ -4175,8 +4529,10 @@
           <t>Ruiz Galeano</t>
         </is>
       </c>
-      <c r="E187" t="n">
-        <v/>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="188">
@@ -4195,8 +4551,10 @@
           <t>Delgado Restrepo</t>
         </is>
       </c>
-      <c r="E188" t="n">
-        <v/>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="189">
@@ -4215,8 +4573,10 @@
           <t>Rodriguez</t>
         </is>
       </c>
-      <c r="E189" t="n">
-        <v/>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="190">
@@ -4235,8 +4595,10 @@
           <t>Zanoja</t>
         </is>
       </c>
-      <c r="E190" t="n">
-        <v/>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="191">
@@ -4255,8 +4617,10 @@
           <t>Cifuentes Gonzalez</t>
         </is>
       </c>
-      <c r="E191" t="n">
-        <v/>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="192">
@@ -4275,8 +4639,10 @@
           <t>Lozano</t>
         </is>
       </c>
-      <c r="E192" t="n">
-        <v/>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="193">
@@ -4295,8 +4661,10 @@
           <t>Guzmán Gomez</t>
         </is>
       </c>
-      <c r="E193" t="n">
-        <v/>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="194">
@@ -4315,8 +4683,10 @@
           <t>Salgdo</t>
         </is>
       </c>
-      <c r="E194" t="n">
-        <v/>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="195">
@@ -4335,8 +4705,10 @@
           <t>Mesa Martínez</t>
         </is>
       </c>
-      <c r="E195" t="n">
-        <v/>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="196">
@@ -4355,8 +4727,10 @@
           <t>Rodríguez</t>
         </is>
       </c>
-      <c r="E196" t="n">
-        <v/>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="197">
@@ -4375,8 +4749,10 @@
           <t>Soto Aristizabal</t>
         </is>
       </c>
-      <c r="E197" t="n">
-        <v/>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="198">
@@ -4395,8 +4771,10 @@
           <t>Velasquez</t>
         </is>
       </c>
-      <c r="E198" t="n">
-        <v/>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="199">
@@ -4415,8 +4793,10 @@
           <t>Agudelo Vélez</t>
         </is>
       </c>
-      <c r="E199" t="n">
-        <v/>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="200">
@@ -4435,8 +4815,10 @@
           <t>León Cruz</t>
         </is>
       </c>
-      <c r="E200" t="n">
-        <v/>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="201">
@@ -4455,8 +4837,10 @@
           <t>Patiño Avendaño</t>
         </is>
       </c>
-      <c r="E201" t="n">
-        <v/>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="202">
@@ -4475,8 +4859,10 @@
           <t>Martínez Giraldo</t>
         </is>
       </c>
-      <c r="E202" t="n">
-        <v/>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="203">
@@ -4495,8 +4881,10 @@
           <t>Calle Echavarria</t>
         </is>
       </c>
-      <c r="E203" t="n">
-        <v/>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="204">
@@ -4515,8 +4903,10 @@
           <t>Rivas Durango</t>
         </is>
       </c>
-      <c r="E204" t="n">
-        <v/>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="205">
@@ -4535,8 +4925,10 @@
           <t>Cabrera</t>
         </is>
       </c>
-      <c r="E205" t="n">
-        <v/>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="206">
@@ -4555,8 +4947,10 @@
           <t>Parada</t>
         </is>
       </c>
-      <c r="E206" t="n">
-        <v/>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="207">
@@ -4575,8 +4969,10 @@
           <t>Fernández Echeverri</t>
         </is>
       </c>
-      <c r="E207" t="n">
-        <v/>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="208">
@@ -4595,8 +4991,10 @@
           <t>Cicery</t>
         </is>
       </c>
-      <c r="E208" t="n">
-        <v/>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="209">
@@ -4615,8 +5013,10 @@
           <t>Jimenez Castañeda</t>
         </is>
       </c>
-      <c r="E209" t="n">
-        <v/>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="210">
@@ -4635,8 +5035,10 @@
           <t>Salamanca Castro</t>
         </is>
       </c>
-      <c r="E210" t="n">
-        <v/>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="211">
@@ -4655,8 +5057,10 @@
           <t>Sanchez Alvarez</t>
         </is>
       </c>
-      <c r="E211" t="n">
-        <v/>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="212">
@@ -4675,8 +5079,10 @@
           <t>Delgado</t>
         </is>
       </c>
-      <c r="E212" t="n">
-        <v/>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="213">
@@ -4695,8 +5101,10 @@
           <t>Rojas Guevara</t>
         </is>
       </c>
-      <c r="E213" t="n">
-        <v/>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="214">
@@ -4715,8 +5123,10 @@
           <t>Martinez</t>
         </is>
       </c>
-      <c r="E214" t="n">
-        <v/>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="215">
@@ -4735,8 +5145,10 @@
           <t>Jiménez</t>
         </is>
       </c>
-      <c r="E215" t="n">
-        <v/>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="216">
@@ -4755,8 +5167,10 @@
           <t>Arias Perez</t>
         </is>
       </c>
-      <c r="E216" t="n">
-        <v/>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="217">
@@ -4775,8 +5189,10 @@
           <t>Salinas</t>
         </is>
       </c>
-      <c r="E217" t="n">
-        <v/>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="218">
@@ -4795,8 +5211,10 @@
           <t>Aristizabal</t>
         </is>
       </c>
-      <c r="E218" t="n">
-        <v/>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="219">
@@ -4815,8 +5233,10 @@
           <t>Serna</t>
         </is>
       </c>
-      <c r="E219" t="n">
-        <v/>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="220">
@@ -4835,8 +5255,10 @@
           <t>Andres Cardona</t>
         </is>
       </c>
-      <c r="E220" t="n">
-        <v/>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="221">
@@ -4855,8 +5277,10 @@
           <t>Callejas Varela</t>
         </is>
       </c>
-      <c r="E221" t="n">
-        <v/>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="222">
@@ -4875,8 +5299,10 @@
           <t>Miranda</t>
         </is>
       </c>
-      <c r="E222" t="n">
-        <v/>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="223">
@@ -4895,8 +5321,10 @@
           <t>Florez Urrego</t>
         </is>
       </c>
-      <c r="E223" t="n">
-        <v/>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="224">
@@ -4915,8 +5343,10 @@
           <t>Cañón</t>
         </is>
       </c>
-      <c r="E224" t="n">
-        <v/>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="225">
@@ -4935,8 +5365,10 @@
           <t>Osorio Tamayo</t>
         </is>
       </c>
-      <c r="E225" t="n">
-        <v/>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="226">
@@ -4955,8 +5387,10 @@
           <t>Lopez</t>
         </is>
       </c>
-      <c r="E226" t="n">
-        <v/>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="227">
@@ -4975,8 +5409,10 @@
           <t>Ceballos</t>
         </is>
       </c>
-      <c r="E227" t="n">
-        <v/>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="228">
@@ -4995,8 +5431,10 @@
           <t>Cristancho</t>
         </is>
       </c>
-      <c r="E228" t="n">
-        <v/>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="229">
@@ -5015,8 +5453,10 @@
           <t>Arias</t>
         </is>
       </c>
-      <c r="E229" t="n">
-        <v/>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="230">
@@ -5035,8 +5475,10 @@
           <t>Arias Cadavid</t>
         </is>
       </c>
-      <c r="E230" t="n">
-        <v/>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="231">
@@ -5055,8 +5497,10 @@
           <t>Zuñiga</t>
         </is>
       </c>
-      <c r="E231" t="n">
-        <v/>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="232">
@@ -5075,8 +5519,10 @@
           <t>Cardona</t>
         </is>
       </c>
-      <c r="E232" t="n">
-        <v/>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="233">
@@ -5095,8 +5541,10 @@
           <t>Clavijo</t>
         </is>
       </c>
-      <c r="E233" t="n">
-        <v/>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="234">
@@ -5115,8 +5563,10 @@
           <t>Torres</t>
         </is>
       </c>
-      <c r="E234" t="n">
-        <v/>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="235">
@@ -5135,8 +5585,10 @@
           <t>Bohórquez</t>
         </is>
       </c>
-      <c r="E235" t="n">
-        <v/>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="236">
@@ -5155,8 +5607,10 @@
           <t>Sierra</t>
         </is>
       </c>
-      <c r="E236" t="n">
-        <v/>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="237">
@@ -5175,8 +5629,10 @@
           <t>Restrepo</t>
         </is>
       </c>
-      <c r="E237" t="n">
-        <v/>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="238">
@@ -5195,8 +5651,10 @@
           <t>Salas</t>
         </is>
       </c>
-      <c r="E238" t="n">
-        <v/>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="239">
@@ -5215,8 +5673,10 @@
           <t>Franco</t>
         </is>
       </c>
-      <c r="E239" t="n">
-        <v/>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="240">
@@ -5235,8 +5695,10 @@
           <t>Garcia Rios</t>
         </is>
       </c>
-      <c r="E240" t="n">
-        <v/>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="241">
@@ -5255,8 +5717,10 @@
           <t>Cecilia Perez Pulgarin</t>
         </is>
       </c>
-      <c r="E241" t="n">
-        <v/>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="242">
@@ -5275,8 +5739,10 @@
           <t>Fabricio Concejal</t>
         </is>
       </c>
-      <c r="E242" t="n">
-        <v/>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="243">
@@ -5295,8 +5761,10 @@
           <t>Humana</t>
         </is>
       </c>
-      <c r="E243" t="n">
-        <v/>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="244">
@@ -5315,8 +5783,10 @@
           <t>Sucerquia</t>
         </is>
       </c>
-      <c r="E244" t="n">
-        <v/>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="245">
@@ -5335,8 +5805,10 @@
           <t>Cabrales</t>
         </is>
       </c>
-      <c r="E245" t="n">
-        <v/>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="246">
@@ -5355,8 +5827,10 @@
           <t>Pasos</t>
         </is>
       </c>
-      <c r="E246" t="n">
-        <v/>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="247">
@@ -5375,8 +5849,10 @@
           <t>González</t>
         </is>
       </c>
-      <c r="E247" t="n">
-        <v/>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="248">
@@ -5395,8 +5871,10 @@
           <t>Salas Araque</t>
         </is>
       </c>
-      <c r="E248" t="n">
-        <v/>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="249">
@@ -5415,8 +5893,10 @@
           <t>Chaparro</t>
         </is>
       </c>
-      <c r="E249" t="n">
-        <v/>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="250">
@@ -5435,8 +5915,10 @@
           <t>Zapata</t>
         </is>
       </c>
-      <c r="E250" t="n">
-        <v/>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="251">
@@ -5455,8 +5937,10 @@
           <t>Morales Cañón</t>
         </is>
       </c>
-      <c r="E251" t="n">
-        <v/>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="252">
@@ -5475,8 +5959,10 @@
           <t>Plazas Sanchez</t>
         </is>
       </c>
-      <c r="E252" t="n">
-        <v/>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="253">
@@ -5495,8 +5981,10 @@
           <t>Agudelo</t>
         </is>
       </c>
-      <c r="E253" t="n">
-        <v/>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="254">
@@ -5515,8 +6003,10 @@
           <t>Adolfo Santa</t>
         </is>
       </c>
-      <c r="E254" t="n">
-        <v/>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="255">
@@ -5535,8 +6025,10 @@
           <t>Medina</t>
         </is>
       </c>
-      <c r="E255" t="n">
-        <v/>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="256">
@@ -5555,8 +6047,10 @@
           <t>Puello</t>
         </is>
       </c>
-      <c r="E256" t="n">
-        <v/>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="257">
@@ -5575,8 +6069,10 @@
           <t>Gutiérrez</t>
         </is>
       </c>
-      <c r="E257" t="n">
-        <v/>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="258">
@@ -5595,8 +6091,10 @@
           <t>Castillo</t>
         </is>
       </c>
-      <c r="E258" t="n">
-        <v/>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="259">
@@ -5615,8 +6113,10 @@
           <t>Bedoya</t>
         </is>
       </c>
-      <c r="E259" t="n">
-        <v/>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="260">
@@ -5657,8 +6157,10 @@
           <t>Rudas</t>
         </is>
       </c>
-      <c r="E261" t="n">
-        <v/>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="262">
@@ -5677,8 +6179,10 @@
           <t>Rodriguez</t>
         </is>
       </c>
-      <c r="E262" t="n">
-        <v/>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="263">
@@ -5697,8 +6201,10 @@
           <t>Vallejo</t>
         </is>
       </c>
-      <c r="E263" t="n">
-        <v/>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="264">
@@ -5717,8 +6223,10 @@
           <t>Perez Sierra</t>
         </is>
       </c>
-      <c r="E264" t="n">
-        <v/>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="265">
@@ -5737,8 +6245,10 @@
           <t>Yepes</t>
         </is>
       </c>
-      <c r="E265" t="n">
-        <v/>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="266">
@@ -5757,8 +6267,10 @@
           <t>Pérez Uribe</t>
         </is>
       </c>
-      <c r="E266" t="n">
-        <v/>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="267">
@@ -5799,8 +6311,10 @@
           <t>Maya G</t>
         </is>
       </c>
-      <c r="E268" t="n">
-        <v/>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="269">
@@ -5819,8 +6333,10 @@
           <t>Rivera Caro</t>
         </is>
       </c>
-      <c r="E269" t="n">
-        <v/>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="270">
@@ -5839,8 +6355,10 @@
           <t>Zapata</t>
         </is>
       </c>
-      <c r="E270" t="n">
-        <v/>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="271">
@@ -5859,8 +6377,10 @@
           <t>Rios</t>
         </is>
       </c>
-      <c r="E271" t="n">
-        <v/>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="272">
@@ -5879,8 +6399,10 @@
           <t>Sandoval</t>
         </is>
       </c>
-      <c r="E272" t="n">
-        <v/>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="273">
@@ -5899,8 +6421,10 @@
           <t>Rodriguez</t>
         </is>
       </c>
-      <c r="E273" t="n">
-        <v/>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="274">
@@ -5919,8 +6443,10 @@
           <t>Alexandra Grisales Vahos</t>
         </is>
       </c>
-      <c r="E274" t="n">
-        <v/>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="275">
@@ -5939,8 +6465,10 @@
           <t>Rhenals Garrido</t>
         </is>
       </c>
-      <c r="E275" t="n">
-        <v/>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="276">
@@ -5959,8 +6487,10 @@
           <t>Gaviria</t>
         </is>
       </c>
-      <c r="E276" t="n">
-        <v/>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="277">
@@ -5979,8 +6509,10 @@
           <t>Ángel</t>
         </is>
       </c>
-      <c r="E277" t="n">
-        <v/>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="278">
@@ -5999,8 +6531,10 @@
           <t>Ayala Lopez</t>
         </is>
       </c>
-      <c r="E278" t="n">
-        <v/>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="279">
@@ -6019,8 +6553,10 @@
           <t>Arango</t>
         </is>
       </c>
-      <c r="E279" t="n">
-        <v/>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="280">
@@ -6039,8 +6575,10 @@
           <t>Campos</t>
         </is>
       </c>
-      <c r="E280" t="n">
-        <v/>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="281">
@@ -6059,8 +6597,10 @@
           <t>Vásquez Rodriguez</t>
         </is>
       </c>
-      <c r="E281" t="n">
-        <v/>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="282">
@@ -6079,8 +6619,10 @@
           <t>Quintero Duque</t>
         </is>
       </c>
-      <c r="E282" t="n">
-        <v/>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="283">
@@ -6099,8 +6641,10 @@
           <t>Restrepo</t>
         </is>
       </c>
-      <c r="E283" t="n">
-        <v/>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="284">
@@ -6119,8 +6663,10 @@
           <t>Ramirez</t>
         </is>
       </c>
-      <c r="E284" t="n">
-        <v/>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="285">
@@ -6139,8 +6685,10 @@
           <t>Muñoz Valero</t>
         </is>
       </c>
-      <c r="E285" t="n">
-        <v/>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="286">
@@ -6159,8 +6707,10 @@
           <t>Cortes</t>
         </is>
       </c>
-      <c r="E286" t="n">
-        <v/>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="287">
@@ -6179,8 +6729,10 @@
           <t>Machado Román</t>
         </is>
       </c>
-      <c r="E287" t="n">
-        <v/>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="288">
@@ -6199,8 +6751,10 @@
           <t>Flórez</t>
         </is>
       </c>
-      <c r="E288" t="n">
-        <v/>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="289">
@@ -6219,8 +6773,10 @@
           <t>Palacio Montoya</t>
         </is>
       </c>
-      <c r="E289" t="n">
-        <v/>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="290">
@@ -6239,8 +6795,10 @@
           <t>Ramirez Sanchez</t>
         </is>
       </c>
-      <c r="E290" t="n">
-        <v/>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="291">
@@ -6259,8 +6817,10 @@
           <t>Hernandez</t>
         </is>
       </c>
-      <c r="E291" t="n">
-        <v/>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="292">
@@ -6279,8 +6839,10 @@
           <t>Castano</t>
         </is>
       </c>
-      <c r="E292" t="n">
-        <v/>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="293">
@@ -6299,8 +6861,10 @@
           <t>Suarez Triana</t>
         </is>
       </c>
-      <c r="E293" t="n">
-        <v/>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="294">
@@ -6319,8 +6883,10 @@
           <t>Ocampo</t>
         </is>
       </c>
-      <c r="E294" t="n">
-        <v/>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="295">
@@ -6339,8 +6905,10 @@
           <t>Ramírez Villegas</t>
         </is>
       </c>
-      <c r="E295" t="n">
-        <v/>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="296">
@@ -6359,8 +6927,10 @@
           <t>Barrios</t>
         </is>
       </c>
-      <c r="E296" t="n">
-        <v/>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="297">
@@ -6379,8 +6949,10 @@
           <t>Sarasa</t>
         </is>
       </c>
-      <c r="E297" t="n">
-        <v/>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="298">
@@ -6399,8 +6971,10 @@
           <t>Meneses</t>
         </is>
       </c>
-      <c r="E298" t="n">
-        <v/>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="299">
@@ -6419,8 +6993,10 @@
           <t>Escobar Franco</t>
         </is>
       </c>
-      <c r="E299" t="n">
-        <v/>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="300">
@@ -6439,8 +7015,10 @@
           <t>Naranjo Pizano</t>
         </is>
       </c>
-      <c r="E300" t="n">
-        <v/>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="301">
@@ -6459,8 +7037,10 @@
           <t>Arboleda</t>
         </is>
       </c>
-      <c r="E301" t="n">
-        <v/>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="302">
@@ -6479,8 +7059,10 @@
           <t>Flórez</t>
         </is>
       </c>
-      <c r="E302" t="n">
-        <v/>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="303">
@@ -6499,8 +7081,10 @@
           <t>Barrera</t>
         </is>
       </c>
-      <c r="E303" t="n">
-        <v/>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="304">
@@ -6519,8 +7103,10 @@
           <t>Alba</t>
         </is>
       </c>
-      <c r="E304" t="n">
-        <v/>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="305">
@@ -6539,8 +7125,10 @@
           <t>Yepes Tabares</t>
         </is>
       </c>
-      <c r="E305" t="n">
-        <v/>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="306">
@@ -6559,8 +7147,10 @@
           <t>Álvarez Restrepo</t>
         </is>
       </c>
-      <c r="E306" t="n">
-        <v/>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="307">
@@ -6579,8 +7169,10 @@
           <t>Payares</t>
         </is>
       </c>
-      <c r="E307" t="n">
-        <v/>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="308">
@@ -6599,8 +7191,10 @@
           <t>Jaramillo</t>
         </is>
       </c>
-      <c r="E308" t="n">
-        <v/>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="309">
@@ -6619,8 +7213,10 @@
           <t>Munera Rua</t>
         </is>
       </c>
-      <c r="E309" t="n">
-        <v/>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="310">
@@ -6639,8 +7235,10 @@
           <t>Alvarez Fernandez</t>
         </is>
       </c>
-      <c r="E310" t="n">
-        <v/>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="311">
@@ -6659,8 +7257,10 @@
           <t>Bedoya</t>
         </is>
       </c>
-      <c r="E311" t="n">
-        <v/>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="312">
@@ -6679,8 +7279,10 @@
           <t>Florez Garcia</t>
         </is>
       </c>
-      <c r="E312" t="n">
-        <v/>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="313">
@@ -6699,8 +7301,10 @@
           <t>Marchese</t>
         </is>
       </c>
-      <c r="E313" t="n">
-        <v/>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="314">
@@ -6719,8 +7323,10 @@
           <t>Prueba Aguilar</t>
         </is>
       </c>
-      <c r="E314" t="n">
-        <v/>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="315">
@@ -6739,8 +7345,10 @@
           <t>Pabon</t>
         </is>
       </c>
-      <c r="E315" t="n">
-        <v/>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="316">
@@ -6759,8 +7367,10 @@
           <t>Or.mm</t>
         </is>
       </c>
-      <c r="E316" t="n">
-        <v/>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="317">
@@ -6779,8 +7389,10 @@
           <t>De La Hoz</t>
         </is>
       </c>
-      <c r="E317" t="n">
-        <v/>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="318">
@@ -6799,8 +7411,10 @@
           <t>Rios</t>
         </is>
       </c>
-      <c r="E318" t="n">
-        <v/>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="319">
@@ -6819,8 +7433,10 @@
           <t>Portilla Araujo</t>
         </is>
       </c>
-      <c r="E319" t="n">
-        <v/>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="320">
@@ -6839,8 +7455,10 @@
           <t>Arango</t>
         </is>
       </c>
-      <c r="E320" t="n">
-        <v/>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
     <row r="321">
@@ -6859,8 +7477,10 @@
           <t>González</t>
         </is>
       </c>
-      <c r="E321" t="n">
-        <v/>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>